<commit_message>
Sending app: the couple send every message from their own WhatsApp
/send installs as its own app. The groom and the bride each log in with
credentials the admin creates, and see their side's guests (a new
"side" column on the guest list, the add form and the upload sheet).
Each guest has one button for the message that is due — invitation,
entry pass, reminder, thank-you — which opens WhatsApp with the approved
template text written out.

A row turns green only when the guest opens the link in the message,
since WhatsApp reports nothing about the send button: the invitation
page, a new /pass and /thanks card page (whose preview image is the
card itself), and a tracked map link in the reminder. Link-preview
fetches don't count. The reminder opens two days before the wedding and
the thank-you the day after, unless the admin sets other dates.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/da3wa-guests-template.xlsx
+++ b/public/da3wa-guests-template.xlsx
@@ -122,10 +122,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -157,10 +157,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -398,12 +398,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D501"/>
+  <dimension ref="A1:E501"/>
   <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="32.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="1" max="1" customWidth="1" width="24.83203125"/>
+    <col min="2" max="2" customWidth="1" width="30.83203125"/>
+    <col min="3" max="3" customWidth="1" width="32.83203125"/>
+    <col min="4" max="4" customWidth="1" width="22.83203125"/>
+    <col min="5" max="5" width="26.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -419,6 +420,9 @@
       <c r="D1" t="str">
         <v>لغة الدعوة (AR أو ENG)</v>
       </c>
+      <c r="E1" t="str">
+        <v>الطرف (العريس أو العروس)</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -433,6 +437,9 @@
       <c r="D2" t="str">
         <v>AR</v>
       </c>
+      <c r="E2" t="str">
+        <v>العريس</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -447,6 +454,9 @@
       <c r="D3" t="str">
         <v>AR</v>
       </c>
+      <c r="E3" t="str">
+        <v>العروس</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -461,6 +471,9 @@
       <c r="D4" t="str">
         <v>ENG</v>
       </c>
+      <c r="E4" t="str">
+        <v>العريس</v>
+      </c>
     </row>
     <row r="5">
       <c r="B5" s="1" t="str">
@@ -2949,7 +2962,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D501"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E501"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>